<commit_message>
feat: Silk-Theme, Fahrgelderstattungs-Generator, Dashboard-Sprungnavigation
- Fahrgelderstattung: Excel/PDF-Generator (ExcelJS + pdf-lib), Stammdaten-Modal,
  bestehendes Dokument hochladen (Konstanten + Unterschrift auto-extrahiert),
  Berufsschultage automatisch aus dem Berichtsheft; bereinigte Firmen-Vorlagen
  (keine Personendaten im Repo).
- Silk-Theme: LightRays-Login-Hintergrund (ogl/WebGL), sanfter Scroll-Parallax,
  Tag-Karten opak statt transluzent, eingeklappte Sidebar (Logo aus, Icons
  zentriert), Dropdown-Menue-Positionierung gefixt.
- Dashboard: Tages-Pills im Hero klickbar -> direkt zum Tag in der Wochenansicht;
  Datums-Badge im Aktuelle-Woche-Hero entfernt.
- Fahrgelderstattung-Seite nutzt die volle Inhaltsbreite.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/fahrgeld-vorlage.xlsx
+++ b/app/templates/fahrgeld-vorlage.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Fahrgelderstattung für Berufsschulbesuche</t>
   </si>
@@ -26,19 +26,7 @@
     <t>Monat / Jahr:</t>
   </si>
   <si>
-    <t>April 26</t>
-  </si>
-  <si>
-    <t>Pers.-Nr.: 101473</t>
-  </si>
-  <si>
     <t>Name, Vorname:</t>
-  </si>
-  <si>
-    <t>Kern, Florian</t>
-  </si>
-  <si>
-    <t>KST: 10000956</t>
   </si>
   <si>
     <t>Datum</t>
@@ -59,12 +47,6 @@
     <t>in €</t>
   </si>
   <si>
-    <t>Grötzingen, Ortsmitte</t>
-  </si>
-  <si>
-    <t>Kirchheim (T) Steingaustraße</t>
-  </si>
-  <si>
     <t>Auszubildender:</t>
   </si>
   <si>
@@ -72,9 +54,6 @@
   </si>
   <si>
     <t>Entgeltabrechnung:</t>
-  </si>
-  <si>
-    <t>26.04.2026</t>
   </si>
   <si>
     <t>Datum / Unterschrift</t>
@@ -665,45 +644,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>344000</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>23999</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1066800" cy="523875"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1035,30 +975,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="11"/>
-      <c r="C4" s="12" t="s">
-        <v>2</v>
-      </c>
+      <c r="C4" s="12"/>
       <c r="D4" s="12"/>
       <c r="E4" s="13"/>
-      <c r="F4" s="11" t="s">
-        <v>3</v>
-      </c>
+      <c r="F4" s="11"/>
       <c r="G4" s="14"/>
       <c r="J4" s="4"/>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="11"/>
-      <c r="C5" s="15" t="s">
-        <v>5</v>
-      </c>
+      <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="13"/>
-      <c r="F5" s="11" t="s">
-        <v>6</v>
-      </c>
+      <c r="F5" s="11"/>
       <c r="G5" s="14"/>
       <c r="J5" s="4"/>
     </row>
@@ -1079,17 +1011,17 @@
     </row>
     <row r="8" ht="27" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="21" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D8" s="22"/>
       <c r="E8" s="22"/>
       <c r="F8" s="20"/>
       <c r="G8" s="23" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4"/>
     </row>
@@ -1097,52 +1029,36 @@
       <c r="A9" s="24"/>
       <c r="B9" s="25"/>
       <c r="C9" s="26" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="28" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F9" s="27"/>
       <c r="G9" s="29" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J9" s="4"/>
     </row>
     <row r="10" ht="24.95" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="30">
-        <v>46124.91666666667</v>
-      </c>
+      <c r="A10" s="30"/>
       <c r="B10" s="31"/>
-      <c r="C10" s="32" t="s">
-        <v>13</v>
-      </c>
+      <c r="C10" s="32"/>
       <c r="D10" s="33"/>
-      <c r="E10" s="32" t="s">
-        <v>14</v>
-      </c>
+      <c r="E10" s="32"/>
       <c r="F10" s="33"/>
-      <c r="G10" s="34">
-        <v>8.3</v>
-      </c>
+      <c r="G10" s="34"/>
       <c r="J10" s="4"/>
     </row>
     <row r="11" ht="24.95" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="30">
-        <v>46132.91666666667</v>
-      </c>
+      <c r="A11" s="30"/>
       <c r="B11" s="35"/>
-      <c r="C11" s="32" t="s">
-        <v>13</v>
-      </c>
+      <c r="C11" s="32"/>
       <c r="D11" s="33"/>
-      <c r="E11" s="32" t="s">
-        <v>14</v>
-      </c>
+      <c r="E11" s="32"/>
       <c r="F11" s="33"/>
-      <c r="G11" s="34">
-        <v>8.3</v>
-      </c>
+      <c r="G11" s="34"/>
       <c r="J11" s="4"/>
     </row>
     <row r="12" ht="24.95" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1227,15 +1143,15 @@
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B20" s="42"/>
       <c r="C20" s="41" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D20" s="42"/>
       <c r="E20" s="41" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="F20" s="42"/>
       <c r="G20" s="43">
@@ -1245,9 +1161,7 @@
       <c r="J20" s="4"/>
     </row>
     <row r="21" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="44" t="s">
-        <v>18</v>
-      </c>
+      <c r="A21" s="44"/>
       <c r="B21" s="45"/>
       <c r="C21" s="44"/>
       <c r="D21" s="45"/>
@@ -1258,25 +1172,25 @@
     </row>
     <row r="22" ht="27" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="47" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B22" s="48"/>
       <c r="C22" s="47" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D22" s="48"/>
       <c r="E22" s="47" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F22" s="48"/>
       <c r="G22" s="49" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="J23" s="4"/>
     </row>

</xml_diff>